<commit_message>
Register Kia Mohave DF100L and prevent Master model confusion
</commit_message>
<xml_diff>
--- a/master-db/kia.xlsx
+++ b/master-db/kia.xlsx
@@ -1385,7 +1385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H153"/>
+  <dimension ref="A1:H154"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5373,6 +5373,48 @@
         <v>12</v>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>모하비</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>19~24년</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>디젤</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>모하비 더 마스터</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>DF100L</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>